<commit_message>
gop lai cac file sheet trong test
</commit_message>
<xml_diff>
--- a/tests/testcase.xlsx
+++ b/tests/testcase.xlsx
@@ -5,18 +5,24 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Study\Nam3\CNPM\FinalProject\lan-may-cafe\tests\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{8395C39A-B28A-460E-BCC6-D5C845873C45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1BAC1910-9F4F-4D2C-9933-D4C518652015}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{7CD00C44-CE7E-4ADA-99E2-520E40CF5D28}"/>
   </bookViews>
   <sheets>
-    <sheet name="Test Case" sheetId="2" r:id="rId1"/>
+    <sheet name="Test Plan" sheetId="3" r:id="rId1"/>
+    <sheet name="Test Case" sheetId="2" r:id="rId2"/>
+    <sheet name="Tổng hợp" sheetId="4" r:id="rId3"/>
+    <sheet name="Bug Report" sheetId="5" r:id="rId4"/>
   </sheets>
+  <externalReferences>
+    <externalReference r:id="rId5"/>
+  </externalReferences>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Test Case'!$A$1:$O$47</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Test Case'!$A$1:$O$47</definedName>
   </definedNames>
   <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
@@ -37,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="585" uniqueCount="368">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="762" uniqueCount="478">
   <si>
     <t>Tên nút theo giao diện của Hậu, cập nhật khi nhận bản 07/10 [X14].</t>
   </si>
@@ -1239,12 +1245,345 @@
   <si>
     <t>ID</t>
   </si>
+  <si>
+    <t>Critical và High: dev sửa trong ngày nhận (Tuấn T8, An A8, Hậu H5). Medium/Low chưa kịp sửa thì chuyển Duy đưa vào mục "Hướng phát triển".</t>
+  </si>
+  <si>
+    <t>Hạn sửa bug</t>
+  </si>
+  <si>
+    <t>Critical: sai tiền, thu trùng, mất hoặc hỏng dữ liệu. High: ảnh hưởng trực tiếp nghiệp vụ hoặc thiếu xử lý alternative flow (ví dụ gọi được món đã hết). Medium: sai thông báo hoặc mã lỗi nhưng nghiệp vụ vẫn đúng. Low: lỗi giao diện, chính tả.</t>
+  </si>
+  <si>
+    <t>Mức độ nghiêm trọng bug</t>
+  </si>
+  <si>
+    <t>Cao: luồng chính, biên, alternative flow quan trọng. Trung: negative/alternative còn lại. Thấp: ít ảnh hưởng nghiệp vụ.</t>
+  </si>
+  <si>
+    <t>Ưu tiên chạy</t>
+  </si>
+  <si>
+    <t>TC-[số UC]-[số thứ tự], ví dụ TC-01-03. Bug: BUG-N5-[số], ví dụ BUG-N5-001. Số UC theo UC diagram cuối (UC01–UC25).</t>
+  </si>
+  <si>
+    <t>Mã test case / bug</t>
+  </si>
+  <si>
+    <t>Quy ước</t>
+  </si>
+  <si>
+    <t>TC thanh toán (UC10), sửa/hủy món (UC04) làm thay đổi dữ liệu: mỗi TC cần đơn còn nguyên, nên chạy reset_db giữa các TC hoặc tạo đơn mới bằng UC01. TC-21-07 khóa tài khoản [TK_PV] nên reset_db sau đó. Nếu thiếu thời gian, chạy các TC ưu tiên "Cao" trước.</t>
+  </si>
+  <si>
+    <t>Lưu ý khi chạy</t>
+  </si>
+  <si>
+    <t>Mỗi TC FAIL viết 1 bug ở sheet "Bug Report" với đủ 7 trường C6-D2; gửi Tuấn, An, Hậu trong ngày 08/10.</t>
+  </si>
+  <si>
+    <t>Bước 3 – Bug report</t>
+  </si>
+  <si>
+    <t>Làm đúng từng bước, không bỏ bước. Ghi Actual Result đúng như quan sát được, không ghi điều bạn nghĩ sẽ xảy ra. Khớp Expected hoàn toàn: PASS; khác ở bất kỳ điểm nào: FAIL. Chụp ảnh bằng chứng, ghi tên file vào cột "Ảnh bằng chứng".</t>
+  </si>
+  <si>
+    <t>Bước 2 – Chạy từng TC</t>
+  </si>
+  <si>
+    <t>Chạy reset_db (script của An) để đưa CSDL về trạng thái ban đầu trước mỗi nhóm test. Ghi lại phiên bản ứng dụng và CSDL ở mục 3. Điền giá trị thật cho các ký hiệu [..] ở sheet "Dữ liệu test".</t>
+  </si>
+  <si>
+    <t>Bước 1 – Chuẩn bị dữ liệu</t>
+  </si>
+  <si>
+    <t>Quy trình thực hiện (theo C6-D2)</t>
+  </si>
+  <si>
+    <t>"Phi chức năng": kiểm tra ngoài luồng UC (ví dụ giao diện chống bấm 2 lần)</t>
+  </si>
+  <si>
+    <t>Không bắt buộc</t>
+  </si>
+  <si>
+    <t>Loại bổ sung</t>
+  </si>
+  <si>
+    <t>Black-box theo UC Specification</t>
+  </si>
+  <si>
+    <t>1 / alternative flow trong UC Spec</t>
+  </si>
+  <si>
+    <t>Boundary Value Analysis</t>
+  </si>
+  <si>
+    <t>2</t>
+  </si>
+  <si>
+    <t>Boundary value</t>
+  </si>
+  <si>
+    <t>Equivalence Partitioning (invalid class)</t>
+  </si>
+  <si>
+    <t>Negative, invalid input</t>
+  </si>
+  <si>
+    <t>Functional test cơ bản</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>Happy path (main flow)</t>
+  </si>
+  <si>
+    <t>Kỹ thuật áp dụng</t>
+  </si>
+  <si>
+    <t>Số lượng tối thiểu / UC</t>
+  </si>
+  <si>
+    <t>Loại test case</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Số test case tối thiểu cho mỗi UC </t>
+  </si>
+  <si>
+    <t>Kiệt – 08/10/2026 (K3); retest 09/10/2026 (K4)</t>
+  </si>
+  <si>
+    <t>Người chạy / ngày chạy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Postman (gọi API), MySQL Workbench (kiểm tra dữ liệu), trình duyệt: ghi tên và phiên bản: </t>
+  </si>
+  <si>
+    <t>Công cụ</t>
+  </si>
+  <si>
+    <t>Node.js &gt;= 18; MySQL 8; server chạy tại http://localhost:3000 (API: http://localhost:3000/api)</t>
+  </si>
+  <si>
+    <t>Nền tảng</t>
+  </si>
+  <si>
+    <t xml:space="preserve">schema.sql + seed.sql của An (nhận 21:00 04/10/2026) – ghi phiên bản hoặc commit: </t>
+  </si>
+  <si>
+    <t>Phiên bản CSDL / seed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">v1.0-rc (nhận 21:00 07/10/2026) – ghi tag và commit hash: </t>
+  </si>
+  <si>
+    <t>Phiên bản ứng dụng</t>
+  </si>
+  <si>
+    <t>Môi trường test (điền khi nhận bản v1.0-rc)</t>
+  </si>
+  <si>
+    <t>Duy</t>
+  </si>
+  <si>
+    <t>Hậu</t>
+  </si>
+  <si>
+    <t>Tuấn</t>
+  </si>
+  <si>
+    <t>Thu ngân</t>
+  </si>
+  <si>
+    <t>Lập hóa đơn</t>
+  </si>
+  <si>
+    <t>UC08</t>
+  </si>
+  <si>
+    <t>Xuân An</t>
+  </si>
+  <si>
+    <t>Bếp</t>
+  </si>
+  <si>
+    <t>Đánh dấu hết nguyên liệu</t>
+  </si>
+  <si>
+    <t>UC18</t>
+  </si>
+  <si>
+    <t>Cập nhật trạng thái chế biến</t>
+  </si>
+  <si>
+    <t>UC16</t>
+  </si>
+  <si>
+    <t>Hiển thị danh sách đơn hàng (KDS)</t>
+  </si>
+  <si>
+    <t>UC15</t>
+  </si>
+  <si>
+    <t>Kiệt</t>
+  </si>
+  <si>
+    <t>Thanh toán hóa đơn (UC10.1 tiền mặt, UC10.2 QR giả lập)</t>
+  </si>
+  <si>
+    <t>Phục vụ</t>
+  </si>
+  <si>
+    <t>Cập nhật order (gọi thêm, sửa, hủy món)</t>
+  </si>
+  <si>
+    <t>Tạo và gửi order</t>
+  </si>
+  <si>
+    <t>Tất cả</t>
+  </si>
+  <si>
+    <t>Đăng nhập hệ thống</t>
+  </si>
+  <si>
+    <t>Số TC</t>
+  </si>
+  <si>
+    <t>Viết + chạy test</t>
+  </si>
+  <si>
+    <t>Frontend</t>
+  </si>
+  <si>
+    <t>Backend</t>
+  </si>
+  <si>
+    <t>Actor</t>
+  </si>
+  <si>
+    <t>Tên UC</t>
+  </si>
+  <si>
+    <t>Phạm vi: 8 UC và phân công test (cross-testing: người viết code không tự test)</t>
+  </si>
+  <si>
+    <t>TEST PLAN – Hệ thống quản lý quán cà phê Làn Mây (Nhóm 5)</t>
+  </si>
+  <si>
+    <t>Nhận xét về độ bao phủ</t>
+  </si>
+  <si>
+    <t>Hướng sửa (method / file)</t>
+  </si>
+  <si>
+    <t>Phân tích nguyên nhân</t>
+  </si>
+  <si>
+    <t>Lỗi nghiêm trọng nhất</t>
+  </si>
+  <si>
+    <t>Tổng hợp số liệu</t>
+  </si>
+  <si>
+    <t>3. Khung báo cáo kết quả (mẫu C6-D2), điền ở K4 trước 21:00 09/10</t>
+  </si>
+  <si>
+    <t>Low</t>
+  </si>
+  <si>
+    <t>Medium</t>
+  </si>
+  <si>
+    <t>High</t>
+  </si>
+  <si>
+    <t>Critical</t>
+  </si>
+  <si>
+    <t>Chưa sửa</t>
+  </si>
+  <si>
+    <t>Đã sửa</t>
+  </si>
+  <si>
+    <t>Số bug</t>
+  </si>
+  <si>
+    <t>Mức độ</t>
+  </si>
+  <si>
+    <t>2. Bug theo mức độ nghiêm trọng</t>
+  </si>
+  <si>
+    <t>FAIL</t>
+  </si>
+  <si>
+    <t>PASS</t>
+  </si>
+  <si>
+    <t>Tổng TC</t>
+  </si>
+  <si>
+    <t>1. Theo loại test case</t>
+  </si>
+  <si>
+    <t>Toàn nhóm (8 UC)</t>
+  </si>
+  <si>
+    <t>TỔNG</t>
+  </si>
+  <si>
+    <t>Tỉ lệ pass (%)</t>
+  </si>
+  <si>
+    <t>Đã chạy</t>
+  </si>
+  <si>
+    <t>Người test</t>
+  </si>
+  <si>
+    <t>TỔNG HỢP KẾT QUẢ KIỂM THỬ</t>
+  </si>
+  <si>
+    <t>Kết quả retest</t>
+  </si>
+  <si>
+    <t>Trạng thái</t>
+  </si>
+  <si>
+    <t>Người sửa</t>
+  </si>
+  <si>
+    <t>Mức độ nghiêm trọng</t>
+  </si>
+  <si>
+    <t>Kết quả mong đợi</t>
+  </si>
+  <si>
+    <t>Kết quả thực tế</t>
+  </si>
+  <si>
+    <t>Bước tái hiện</t>
+  </si>
+  <si>
+    <t>Mô tả lỗi</t>
+  </si>
+  <si>
+    <t>Related TC</t>
+  </si>
+  <si>
+    <t>Bug ID</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.0%"/>
+  </numFmts>
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1279,8 +1618,29 @@
       <name val="Arial"/>
       <charset val="1"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Arial"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color rgb="FF1F3864"/>
+      <name val="Arial"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF1F3864"/>
+      <name val="Arial"/>
+      <charset val="1"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1299,8 +1659,20 @@
         <bgColor rgb="FFED7D31"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFDDEBF7"/>
+        <bgColor rgb="FFEDEDED"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF2CC"/>
+        <bgColor rgb="FFEDEDED"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -1323,12 +1695,25 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFBFBFBF"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color rgb="FFBFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFBFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1345,6 +1730,37 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="4" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1401,6 +1817,262 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
+  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+    <xxl21:alternateUrls>
+      <xxl21:absoluteUrl r:id="rId2"/>
+    </xxl21:alternateUrls>
+    <sheetNames>
+      <sheetName val="Dữ liệu test"/>
+      <sheetName val="Test Case"/>
+      <sheetName val="Cần xác nhận"/>
+    </sheetNames>
+    <sheetDataSet>
+      <sheetData sheetId="0"/>
+      <sheetData sheetId="1">
+        <row r="2">
+          <cell r="B2" t="str">
+            <v>UC</v>
+          </cell>
+        </row>
+        <row r="3">
+          <cell r="B3" t="str">
+            <v>UC21</v>
+          </cell>
+        </row>
+        <row r="4">
+          <cell r="B4" t="str">
+            <v>UC21</v>
+          </cell>
+        </row>
+        <row r="5">
+          <cell r="B5" t="str">
+            <v>UC21</v>
+          </cell>
+        </row>
+        <row r="6">
+          <cell r="B6" t="str">
+            <v>UC21</v>
+          </cell>
+        </row>
+        <row r="7">
+          <cell r="B7" t="str">
+            <v>UC21</v>
+          </cell>
+        </row>
+        <row r="8">
+          <cell r="B8" t="str">
+            <v>UC21</v>
+          </cell>
+        </row>
+        <row r="9">
+          <cell r="B9" t="str">
+            <v>UC21</v>
+          </cell>
+        </row>
+        <row r="10">
+          <cell r="B10" t="str">
+            <v>UC21</v>
+          </cell>
+        </row>
+        <row r="11">
+          <cell r="B11" t="str">
+            <v>UC21</v>
+          </cell>
+        </row>
+        <row r="12">
+          <cell r="B12" t="str">
+            <v>UC21</v>
+          </cell>
+        </row>
+        <row r="13">
+          <cell r="B13" t="str">
+            <v>UC21</v>
+          </cell>
+        </row>
+        <row r="14">
+          <cell r="B14" t="str">
+            <v>UC01</v>
+          </cell>
+        </row>
+        <row r="15">
+          <cell r="B15" t="str">
+            <v>UC01</v>
+          </cell>
+        </row>
+        <row r="16">
+          <cell r="B16" t="str">
+            <v>UC01</v>
+          </cell>
+        </row>
+        <row r="17">
+          <cell r="B17" t="str">
+            <v>UC01</v>
+          </cell>
+        </row>
+        <row r="18">
+          <cell r="B18" t="str">
+            <v>UC01</v>
+          </cell>
+        </row>
+        <row r="19">
+          <cell r="B19" t="str">
+            <v>UC01</v>
+          </cell>
+        </row>
+        <row r="20">
+          <cell r="B20" t="str">
+            <v>UC01</v>
+          </cell>
+        </row>
+        <row r="21">
+          <cell r="B21" t="str">
+            <v>UC01</v>
+          </cell>
+        </row>
+        <row r="22">
+          <cell r="B22" t="str">
+            <v>UC01</v>
+          </cell>
+        </row>
+        <row r="23">
+          <cell r="B23" t="str">
+            <v>UC01</v>
+          </cell>
+        </row>
+        <row r="24">
+          <cell r="B24" t="str">
+            <v>UC01</v>
+          </cell>
+        </row>
+        <row r="25">
+          <cell r="B25" t="str">
+            <v>UC04</v>
+          </cell>
+        </row>
+        <row r="26">
+          <cell r="B26" t="str">
+            <v>UC04</v>
+          </cell>
+        </row>
+        <row r="27">
+          <cell r="B27" t="str">
+            <v>UC04</v>
+          </cell>
+        </row>
+        <row r="28">
+          <cell r="B28" t="str">
+            <v>UC04</v>
+          </cell>
+        </row>
+        <row r="29">
+          <cell r="B29" t="str">
+            <v>UC04</v>
+          </cell>
+        </row>
+        <row r="30">
+          <cell r="B30" t="str">
+            <v>UC04</v>
+          </cell>
+        </row>
+        <row r="31">
+          <cell r="B31" t="str">
+            <v>UC04</v>
+          </cell>
+        </row>
+        <row r="32">
+          <cell r="B32" t="str">
+            <v>UC04</v>
+          </cell>
+        </row>
+        <row r="33">
+          <cell r="B33" t="str">
+            <v>UC04</v>
+          </cell>
+        </row>
+        <row r="34">
+          <cell r="B34" t="str">
+            <v>UC04</v>
+          </cell>
+        </row>
+        <row r="35">
+          <cell r="B35" t="str">
+            <v>UC04</v>
+          </cell>
+        </row>
+        <row r="36">
+          <cell r="B36" t="str">
+            <v>UC04</v>
+          </cell>
+        </row>
+        <row r="37">
+          <cell r="B37" t="str">
+            <v>UC04</v>
+          </cell>
+        </row>
+        <row r="38">
+          <cell r="B38" t="str">
+            <v>UC10</v>
+          </cell>
+        </row>
+        <row r="39">
+          <cell r="B39" t="str">
+            <v>UC10</v>
+          </cell>
+        </row>
+        <row r="40">
+          <cell r="B40" t="str">
+            <v>UC10</v>
+          </cell>
+        </row>
+        <row r="41">
+          <cell r="B41" t="str">
+            <v>UC10</v>
+          </cell>
+        </row>
+        <row r="42">
+          <cell r="B42" t="str">
+            <v>UC10</v>
+          </cell>
+        </row>
+        <row r="43">
+          <cell r="B43" t="str">
+            <v>UC10</v>
+          </cell>
+        </row>
+        <row r="44">
+          <cell r="B44" t="str">
+            <v>UC10</v>
+          </cell>
+        </row>
+        <row r="45">
+          <cell r="B45" t="str">
+            <v>UC10</v>
+          </cell>
+        </row>
+        <row r="46">
+          <cell r="B46" t="str">
+            <v>UC10</v>
+          </cell>
+        </row>
+        <row r="47">
+          <cell r="B47" t="str">
+            <v>UC10</v>
+          </cell>
+        </row>
+        <row r="48">
+          <cell r="B48" t="str">
+            <v>UC10</v>
+          </cell>
+        </row>
+      </sheetData>
+      <sheetData sheetId="2"/>
+    </sheetDataSet>
+  </externalBook>
+</externalLink>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1699,6 +2371,584 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{689663C2-C013-4EAA-A00B-255D1FF81DD9}">
+  <sheetPr>
+    <tabColor rgb="FF1F3864"/>
+  </sheetPr>
+  <dimension ref="A1:G39"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="26" style="1" customWidth="1"/>
+    <col min="2" max="2" width="36" style="1" customWidth="1"/>
+    <col min="3" max="3" width="16" style="1" customWidth="1"/>
+    <col min="4" max="5" width="14" style="1" customWidth="1"/>
+    <col min="6" max="6" width="26" style="1" customWidth="1"/>
+    <col min="7" max="7" width="12" style="1" customWidth="1"/>
+    <col min="8" max="16384" width="8.7109375" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" ht="18" x14ac:dyDescent="0.25">
+      <c r="A1" s="13" t="s">
+        <v>442</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" s="10" t="s">
+        <v>441</v>
+      </c>
+      <c r="B3" s="9"/>
+      <c r="C3" s="9"/>
+      <c r="D3" s="9"/>
+      <c r="E3" s="9"/>
+      <c r="F3" s="9"/>
+      <c r="G3" s="9"/>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" s="5" t="s">
+        <v>366</v>
+      </c>
+      <c r="B4" s="5" t="s">
+        <v>440</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>439</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>438</v>
+      </c>
+      <c r="E4" s="5" t="s">
+        <v>437</v>
+      </c>
+      <c r="F4" s="5" t="s">
+        <v>436</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>435</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="4" t="s">
+        <v>271</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>434</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>433</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>415</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>415</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>428</v>
+      </c>
+      <c r="G5" s="3" t="e">
+        <f>COUNTIF('[1]Test Case'!$B:$B,A5)</f>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="4" t="s">
+        <v>193</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>432</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>430</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>416</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>415</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>428</v>
+      </c>
+      <c r="G6" s="3" t="e">
+        <f>COUNTIF('[1]Test Case'!$B:$B,A6)</f>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>431</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>430</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>416</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>415</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>428</v>
+      </c>
+      <c r="G7" s="3" t="e">
+        <f>COUNTIF('[1]Test Case'!$B:$B,A7)</f>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>429</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>417</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>416</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>415</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>428</v>
+      </c>
+      <c r="G8" s="3" t="e">
+        <f>COUNTIF('[1]Test Case'!$B:$B,A8)</f>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="4" t="s">
+        <v>427</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>426</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>421</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>420</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>420</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>414</v>
+      </c>
+      <c r="G9" s="3" t="e">
+        <f>COUNTIF('[1]Test Case'!$B:$B,A9)</f>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="4" t="s">
+        <v>425</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>424</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>421</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>420</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>420</v>
+      </c>
+      <c r="F10" s="3" t="s">
+        <v>414</v>
+      </c>
+      <c r="G10" s="3" t="e">
+        <f>COUNTIF('[1]Test Case'!$B:$B,A10)</f>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="4" t="s">
+        <v>423</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>422</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>421</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>420</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>420</v>
+      </c>
+      <c r="F11" s="3" t="s">
+        <v>414</v>
+      </c>
+      <c r="G11" s="3" t="e">
+        <f>COUNTIF('[1]Test Case'!$B:$B,A11)</f>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="4" t="s">
+        <v>419</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>418</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>417</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>416</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>415</v>
+      </c>
+      <c r="F12" s="3" t="s">
+        <v>414</v>
+      </c>
+      <c r="G12" s="3" t="e">
+        <f>COUNTIF('[1]Test Case'!$B:$B,A12)</f>
+        <v>#VALUE!</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A14" s="10" t="s">
+        <v>413</v>
+      </c>
+      <c r="B14" s="9"/>
+      <c r="C14" s="9"/>
+      <c r="D14" s="9"/>
+      <c r="E14" s="9"/>
+      <c r="F14" s="9"/>
+      <c r="G14" s="9"/>
+    </row>
+    <row r="15" spans="1:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="8" t="s">
+        <v>412</v>
+      </c>
+      <c r="B15" s="12" t="s">
+        <v>411</v>
+      </c>
+      <c r="C15" s="12"/>
+      <c r="D15" s="12"/>
+      <c r="E15" s="12"/>
+      <c r="F15" s="12"/>
+      <c r="G15" s="12"/>
+    </row>
+    <row r="16" spans="1:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="8" t="s">
+        <v>410</v>
+      </c>
+      <c r="B16" s="12" t="s">
+        <v>409</v>
+      </c>
+      <c r="C16" s="12"/>
+      <c r="D16" s="12"/>
+      <c r="E16" s="12"/>
+      <c r="F16" s="12"/>
+      <c r="G16" s="12"/>
+    </row>
+    <row r="17" spans="1:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="8" t="s">
+        <v>408</v>
+      </c>
+      <c r="B17" s="7" t="s">
+        <v>407</v>
+      </c>
+      <c r="C17" s="7"/>
+      <c r="D17" s="7"/>
+      <c r="E17" s="7"/>
+      <c r="F17" s="7"/>
+      <c r="G17" s="7"/>
+    </row>
+    <row r="18" spans="1:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="8" t="s">
+        <v>406</v>
+      </c>
+      <c r="B18" s="12" t="s">
+        <v>405</v>
+      </c>
+      <c r="C18" s="12"/>
+      <c r="D18" s="12"/>
+      <c r="E18" s="12"/>
+      <c r="F18" s="12"/>
+      <c r="G18" s="12"/>
+    </row>
+    <row r="19" spans="1:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="8" t="s">
+        <v>404</v>
+      </c>
+      <c r="B19" s="7" t="s">
+        <v>403</v>
+      </c>
+      <c r="C19" s="7"/>
+      <c r="D19" s="7"/>
+      <c r="E19" s="7"/>
+      <c r="F19" s="7"/>
+      <c r="G19" s="7"/>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A21" s="10" t="s">
+        <v>402</v>
+      </c>
+      <c r="B21" s="9"/>
+      <c r="C21" s="9"/>
+      <c r="D21" s="9"/>
+      <c r="E21" s="9"/>
+      <c r="F21" s="9"/>
+      <c r="G21" s="9"/>
+    </row>
+    <row r="22" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A22" s="5" t="s">
+        <v>401</v>
+      </c>
+      <c r="B22" s="5" t="s">
+        <v>400</v>
+      </c>
+      <c r="C22" s="11" t="s">
+        <v>399</v>
+      </c>
+      <c r="D22" s="11"/>
+      <c r="E22" s="11"/>
+      <c r="F22" s="11"/>
+      <c r="G22" s="11"/>
+    </row>
+    <row r="23" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A23" s="8" t="s">
+        <v>398</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>397</v>
+      </c>
+      <c r="C23" s="7" t="s">
+        <v>396</v>
+      </c>
+      <c r="D23" s="7"/>
+      <c r="E23" s="7"/>
+      <c r="F23" s="7"/>
+      <c r="G23" s="7"/>
+    </row>
+    <row r="24" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="8" t="s">
+        <v>395</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>392</v>
+      </c>
+      <c r="C24" s="7" t="s">
+        <v>394</v>
+      </c>
+      <c r="D24" s="7"/>
+      <c r="E24" s="7"/>
+      <c r="F24" s="7"/>
+      <c r="G24" s="7"/>
+    </row>
+    <row r="25" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="8" t="s">
+        <v>393</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>392</v>
+      </c>
+      <c r="C25" s="7" t="s">
+        <v>391</v>
+      </c>
+      <c r="D25" s="7"/>
+      <c r="E25" s="7"/>
+      <c r="F25" s="7"/>
+      <c r="G25" s="7"/>
+    </row>
+    <row r="26" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>390</v>
+      </c>
+      <c r="C26" s="7" t="s">
+        <v>389</v>
+      </c>
+      <c r="D26" s="7"/>
+      <c r="E26" s="7"/>
+      <c r="F26" s="7"/>
+      <c r="G26" s="7"/>
+    </row>
+    <row r="27" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="8" t="s">
+        <v>388</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>387</v>
+      </c>
+      <c r="C27" s="7" t="s">
+        <v>386</v>
+      </c>
+      <c r="D27" s="7"/>
+      <c r="E27" s="7"/>
+      <c r="F27" s="7"/>
+      <c r="G27" s="7"/>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A29" s="10" t="s">
+        <v>385</v>
+      </c>
+      <c r="B29" s="9"/>
+      <c r="C29" s="9"/>
+      <c r="D29" s="9"/>
+      <c r="E29" s="9"/>
+      <c r="F29" s="9"/>
+      <c r="G29" s="9"/>
+    </row>
+    <row r="30" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="8" t="s">
+        <v>384</v>
+      </c>
+      <c r="B30" s="7" t="s">
+        <v>383</v>
+      </c>
+      <c r="C30" s="7"/>
+      <c r="D30" s="7"/>
+      <c r="E30" s="7"/>
+      <c r="F30" s="7"/>
+      <c r="G30" s="7"/>
+    </row>
+    <row r="31" spans="1:7" ht="43.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="8" t="s">
+        <v>382</v>
+      </c>
+      <c r="B31" s="7" t="s">
+        <v>381</v>
+      </c>
+      <c r="C31" s="7"/>
+      <c r="D31" s="7"/>
+      <c r="E31" s="7"/>
+      <c r="F31" s="7"/>
+      <c r="G31" s="7"/>
+    </row>
+    <row r="32" spans="1:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="8" t="s">
+        <v>380</v>
+      </c>
+      <c r="B32" s="7" t="s">
+        <v>379</v>
+      </c>
+      <c r="C32" s="7"/>
+      <c r="D32" s="7"/>
+      <c r="E32" s="7"/>
+      <c r="F32" s="7"/>
+      <c r="G32" s="7"/>
+    </row>
+    <row r="33" spans="1:7" ht="43.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="8" t="s">
+        <v>378</v>
+      </c>
+      <c r="B33" s="7" t="s">
+        <v>377</v>
+      </c>
+      <c r="C33" s="7"/>
+      <c r="D33" s="7"/>
+      <c r="E33" s="7"/>
+      <c r="F33" s="7"/>
+      <c r="G33" s="7"/>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A35" s="10" t="s">
+        <v>376</v>
+      </c>
+      <c r="B35" s="9"/>
+      <c r="C35" s="9"/>
+      <c r="D35" s="9"/>
+      <c r="E35" s="9"/>
+      <c r="F35" s="9"/>
+      <c r="G35" s="9"/>
+    </row>
+    <row r="36" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A36" s="8" t="s">
+        <v>375</v>
+      </c>
+      <c r="B36" s="7" t="s">
+        <v>374</v>
+      </c>
+      <c r="C36" s="7"/>
+      <c r="D36" s="7"/>
+      <c r="E36" s="7"/>
+      <c r="F36" s="7"/>
+      <c r="G36" s="7"/>
+    </row>
+    <row r="37" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A37" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="B37" s="7" t="s">
+        <v>372</v>
+      </c>
+      <c r="C37" s="7"/>
+      <c r="D37" s="7"/>
+      <c r="E37" s="7"/>
+      <c r="F37" s="7"/>
+      <c r="G37" s="7"/>
+    </row>
+    <row r="38" spans="1:7" ht="43.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A38" s="8" t="s">
+        <v>371</v>
+      </c>
+      <c r="B38" s="7" t="s">
+        <v>370</v>
+      </c>
+      <c r="C38" s="7"/>
+      <c r="D38" s="7"/>
+      <c r="E38" s="7"/>
+      <c r="F38" s="7"/>
+      <c r="G38" s="7"/>
+    </row>
+    <row r="39" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A39" s="8" t="s">
+        <v>369</v>
+      </c>
+      <c r="B39" s="7" t="s">
+        <v>368</v>
+      </c>
+      <c r="C39" s="7"/>
+      <c r="D39" s="7"/>
+      <c r="E39" s="7"/>
+      <c r="F39" s="7"/>
+      <c r="G39" s="7"/>
+    </row>
+  </sheetData>
+  <mergeCells count="19">
+    <mergeCell ref="B37:G37"/>
+    <mergeCell ref="B38:G38"/>
+    <mergeCell ref="B39:G39"/>
+    <mergeCell ref="C24:G24"/>
+    <mergeCell ref="C25:G25"/>
+    <mergeCell ref="C26:G26"/>
+    <mergeCell ref="C27:G27"/>
+    <mergeCell ref="B30:G30"/>
+    <mergeCell ref="B31:G31"/>
+    <mergeCell ref="B32:G32"/>
+    <mergeCell ref="B33:G33"/>
+    <mergeCell ref="B36:G36"/>
+    <mergeCell ref="C23:G23"/>
+    <mergeCell ref="B15:G15"/>
+    <mergeCell ref="B16:G16"/>
+    <mergeCell ref="B17:G17"/>
+    <mergeCell ref="B18:G18"/>
+    <mergeCell ref="B19:G19"/>
+    <mergeCell ref="C22:G22"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A6038F87-EB00-45B1-AC25-57ADB6A4FABB}">
   <sheetPr>
     <tabColor rgb="FF2E75B6"/>
@@ -3723,4 +4973,619 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EF16DF64-E532-43F9-A54C-6B964E0DDE89}">
+  <sheetPr>
+    <tabColor rgb="FF548235"/>
+  </sheetPr>
+  <dimension ref="A1:J35"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="18" style="1" customWidth="1"/>
+    <col min="2" max="2" width="44" style="1" customWidth="1"/>
+    <col min="3" max="3" width="14" style="1" customWidth="1"/>
+    <col min="4" max="8" width="12" style="1" customWidth="1"/>
+    <col min="9" max="9" width="16" style="1" customWidth="1"/>
+    <col min="10" max="10" width="12" style="1" customWidth="1"/>
+    <col min="11" max="16384" width="8.7109375" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10" ht="18" x14ac:dyDescent="0.25">
+      <c r="A1" s="13" t="s">
+        <v>467</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="5" t="s">
+        <v>366</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>440</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>466</v>
+      </c>
+      <c r="D3" s="5" t="s">
+        <v>460</v>
+      </c>
+      <c r="E3" s="5" t="s">
+        <v>465</v>
+      </c>
+      <c r="F3" s="5" t="s">
+        <v>459</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>458</v>
+      </c>
+      <c r="H3" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="I3" s="5" t="s">
+        <v>464</v>
+      </c>
+      <c r="J3" s="5" t="s">
+        <v>455</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A4" s="4" t="s">
+        <v>271</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>434</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>428</v>
+      </c>
+      <c r="D4" s="3"/>
+      <c r="E4" s="3"/>
+      <c r="F4" s="3"/>
+      <c r="G4" s="3"/>
+      <c r="H4" s="3"/>
+      <c r="I4" s="19"/>
+      <c r="J4" s="3">
+        <f>COUNTIFS('Bug Report'!$A:$A,"BUG-N5-*",'Bug Report'!$B:$B,"TC-"&amp;RIGHT($A4,2)&amp;"-*")</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A5" s="4" t="s">
+        <v>193</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>432</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>428</v>
+      </c>
+      <c r="D5" s="3"/>
+      <c r="E5" s="3"/>
+      <c r="F5" s="3"/>
+      <c r="G5" s="3"/>
+      <c r="H5" s="3"/>
+      <c r="I5" s="19"/>
+      <c r="J5" s="3">
+        <f>COUNTIFS('Bug Report'!$A:$A,"BUG-N5-*",'Bug Report'!$B:$B,"TC-"&amp;RIGHT($A5,2)&amp;"-*")</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A6" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>431</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>428</v>
+      </c>
+      <c r="D6" s="3"/>
+      <c r="E6" s="3"/>
+      <c r="F6" s="3"/>
+      <c r="G6" s="3"/>
+      <c r="H6" s="3"/>
+      <c r="I6" s="19"/>
+      <c r="J6" s="3">
+        <f>COUNTIFS('Bug Report'!$A:$A,"BUG-N5-*",'Bug Report'!$B:$B,"TC-"&amp;RIGHT($A6,2)&amp;"-*")</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A7" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>429</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>428</v>
+      </c>
+      <c r="D7" s="3"/>
+      <c r="E7" s="3"/>
+      <c r="F7" s="3"/>
+      <c r="G7" s="3"/>
+      <c r="H7" s="3"/>
+      <c r="I7" s="19"/>
+      <c r="J7" s="3">
+        <f>COUNTIFS('Bug Report'!$A:$A,"BUG-N5-*",'Bug Report'!$B:$B,"TC-"&amp;RIGHT($A7,2)&amp;"-*")</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A8" s="4" t="s">
+        <v>427</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>426</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>414</v>
+      </c>
+      <c r="D8" s="3"/>
+      <c r="E8" s="3"/>
+      <c r="F8" s="3"/>
+      <c r="G8" s="3"/>
+      <c r="H8" s="3"/>
+      <c r="I8" s="19"/>
+      <c r="J8" s="3">
+        <f>COUNTIFS('Bug Report'!$A:$A,"BUG-N5-*",'Bug Report'!$B:$B,"TC-"&amp;RIGHT($A8,2)&amp;"-*")</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A9" s="4" t="s">
+        <v>425</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>424</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>414</v>
+      </c>
+      <c r="D9" s="3"/>
+      <c r="E9" s="3"/>
+      <c r="F9" s="3"/>
+      <c r="G9" s="3"/>
+      <c r="H9" s="3"/>
+      <c r="I9" s="19"/>
+      <c r="J9" s="3">
+        <f>COUNTIFS('Bug Report'!$A:$A,"BUG-N5-*",'Bug Report'!$B:$B,"TC-"&amp;RIGHT($A9,2)&amp;"-*")</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A10" s="4" t="s">
+        <v>423</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>422</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>414</v>
+      </c>
+      <c r="D10" s="3"/>
+      <c r="E10" s="3"/>
+      <c r="F10" s="3"/>
+      <c r="G10" s="3"/>
+      <c r="H10" s="3"/>
+      <c r="I10" s="19"/>
+      <c r="J10" s="3">
+        <f>COUNTIFS('Bug Report'!$A:$A,"BUG-N5-*",'Bug Report'!$B:$B,"TC-"&amp;RIGHT($A10,2)&amp;"-*")</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A11" s="4" t="s">
+        <v>419</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>418</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>414</v>
+      </c>
+      <c r="D11" s="3"/>
+      <c r="E11" s="3"/>
+      <c r="F11" s="3"/>
+      <c r="G11" s="3"/>
+      <c r="H11" s="3"/>
+      <c r="I11" s="19"/>
+      <c r="J11" s="3">
+        <f>COUNTIFS('Bug Report'!$A:$A,"BUG-N5-*",'Bug Report'!$B:$B,"TC-"&amp;RIGHT($A11,2)&amp;"-*")</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A12" s="16" t="s">
+        <v>463</v>
+      </c>
+      <c r="B12" s="8" t="s">
+        <v>462</v>
+      </c>
+      <c r="C12" s="18"/>
+      <c r="D12" s="16"/>
+      <c r="E12" s="16"/>
+      <c r="F12" s="16"/>
+      <c r="G12" s="16"/>
+      <c r="H12" s="16"/>
+      <c r="I12" s="17"/>
+      <c r="J12" s="16">
+        <f>SUM(J4:J11)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A14" s="14" t="s">
+        <v>461</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="5" t="s">
+        <v>364</v>
+      </c>
+      <c r="B15" s="5"/>
+      <c r="C15" s="5"/>
+      <c r="D15" s="5" t="s">
+        <v>460</v>
+      </c>
+      <c r="E15" s="5" t="s">
+        <v>459</v>
+      </c>
+      <c r="F15" s="5" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A16" s="15" t="s">
+        <v>54</v>
+      </c>
+      <c r="B16" s="2"/>
+      <c r="C16" s="2"/>
+      <c r="D16" s="3"/>
+      <c r="E16" s="3"/>
+      <c r="F16" s="3"/>
+    </row>
+    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A17" s="15" t="s">
+        <v>62</v>
+      </c>
+      <c r="B17" s="2"/>
+      <c r="C17" s="2"/>
+      <c r="D17" s="3"/>
+      <c r="E17" s="3"/>
+      <c r="F17" s="3"/>
+    </row>
+    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A18" s="15" t="s">
+        <v>78</v>
+      </c>
+      <c r="B18" s="2"/>
+      <c r="C18" s="2"/>
+      <c r="D18" s="3"/>
+      <c r="E18" s="3"/>
+      <c r="F18" s="3"/>
+    </row>
+    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A19" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="B19" s="2"/>
+      <c r="C19" s="2"/>
+      <c r="D19" s="3"/>
+      <c r="E19" s="3"/>
+      <c r="F19" s="3"/>
+    </row>
+    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A20" s="15" t="s">
+        <v>9</v>
+      </c>
+      <c r="B20" s="2"/>
+      <c r="C20" s="2"/>
+      <c r="D20" s="3"/>
+      <c r="E20" s="3"/>
+      <c r="F20" s="3"/>
+    </row>
+    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A23" s="14" t="s">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="5" t="s">
+        <v>456</v>
+      </c>
+      <c r="B24" s="5"/>
+      <c r="C24" s="5"/>
+      <c r="D24" s="5" t="s">
+        <v>455</v>
+      </c>
+      <c r="E24" s="5" t="s">
+        <v>454</v>
+      </c>
+      <c r="F24" s="5" t="s">
+        <v>453</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A25" s="15" t="s">
+        <v>452</v>
+      </c>
+      <c r="B25" s="2"/>
+      <c r="C25" s="2"/>
+      <c r="D25" s="3">
+        <f>COUNTIFS('Bug Report'!$A:$A,"BUG-N5-*",'Bug Report'!$G:$G,$A25)</f>
+        <v>0</v>
+      </c>
+      <c r="E25" s="3">
+        <f>COUNTIFS('Bug Report'!$A:$A,"BUG-N5-*",'Bug Report'!$G:$G,$A25,'Bug Report'!$I:$I,"Đã retest đạt")</f>
+        <v>0</v>
+      </c>
+      <c r="F25" s="3">
+        <f>D25-E25</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A26" s="15" t="s">
+        <v>451</v>
+      </c>
+      <c r="B26" s="2"/>
+      <c r="C26" s="2"/>
+      <c r="D26" s="3">
+        <f>COUNTIFS('Bug Report'!$A:$A,"BUG-N5-*",'Bug Report'!$G:$G,$A26)</f>
+        <v>0</v>
+      </c>
+      <c r="E26" s="3">
+        <f>COUNTIFS('Bug Report'!$A:$A,"BUG-N5-*",'Bug Report'!$G:$G,$A26,'Bug Report'!$I:$I,"Đã retest đạt")</f>
+        <v>0</v>
+      </c>
+      <c r="F26" s="3">
+        <f>D26-E26</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A27" s="15" t="s">
+        <v>450</v>
+      </c>
+      <c r="B27" s="2"/>
+      <c r="C27" s="2"/>
+      <c r="D27" s="3">
+        <f>COUNTIFS('Bug Report'!$A:$A,"BUG-N5-*",'Bug Report'!$G:$G,$A27)</f>
+        <v>0</v>
+      </c>
+      <c r="E27" s="3">
+        <f>COUNTIFS('Bug Report'!$A:$A,"BUG-N5-*",'Bug Report'!$G:$G,$A27,'Bug Report'!$I:$I,"Đã retest đạt")</f>
+        <v>0</v>
+      </c>
+      <c r="F27" s="3">
+        <f>D27-E27</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A28" s="15" t="s">
+        <v>449</v>
+      </c>
+      <c r="B28" s="2"/>
+      <c r="C28" s="2"/>
+      <c r="D28" s="3">
+        <f>COUNTIFS('Bug Report'!$A:$A,"BUG-N5-*",'Bug Report'!$G:$G,$A28)</f>
+        <v>0</v>
+      </c>
+      <c r="E28" s="3">
+        <f>COUNTIFS('Bug Report'!$A:$A,"BUG-N5-*",'Bug Report'!$G:$G,$A28,'Bug Report'!$I:$I,"Đã retest đạt")</f>
+        <v>0</v>
+      </c>
+      <c r="F28" s="3">
+        <f>D28-E28</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A30" s="14" t="s">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="8" t="s">
+        <v>447</v>
+      </c>
+      <c r="B31" s="7" t="str">
+        <f>"Đã chạy "&amp;E12&amp;" / "&amp;D12&amp;" TC; PASS "&amp;F12&amp;"; FAIL "&amp;G12&amp;"; tỉ lệ pass "&amp;IF(E12=0,"-",TEXT(F12/E12,"0.0%"))</f>
+        <v>Đã chạy  /  TC; PASS ; FAIL ; tỉ lệ pass -</v>
+      </c>
+      <c r="C31" s="7"/>
+      <c r="D31" s="7"/>
+      <c r="E31" s="7"/>
+      <c r="F31" s="7"/>
+      <c r="G31" s="7"/>
+      <c r="H31" s="7"/>
+      <c r="I31" s="7"/>
+      <c r="J31" s="7"/>
+    </row>
+    <row r="32" spans="1:10" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="8" t="s">
+        <v>446</v>
+      </c>
+      <c r="B32" s="12"/>
+      <c r="C32" s="12"/>
+      <c r="D32" s="12"/>
+      <c r="E32" s="12"/>
+      <c r="F32" s="12"/>
+      <c r="G32" s="12"/>
+      <c r="H32" s="12"/>
+      <c r="I32" s="12"/>
+      <c r="J32" s="12"/>
+    </row>
+    <row r="33" spans="1:10" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="8" t="s">
+        <v>445</v>
+      </c>
+      <c r="B33" s="12"/>
+      <c r="C33" s="12"/>
+      <c r="D33" s="12"/>
+      <c r="E33" s="12"/>
+      <c r="F33" s="12"/>
+      <c r="G33" s="12"/>
+      <c r="H33" s="12"/>
+      <c r="I33" s="12"/>
+      <c r="J33" s="12"/>
+    </row>
+    <row r="34" spans="1:10" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="8" t="s">
+        <v>444</v>
+      </c>
+      <c r="B34" s="12"/>
+      <c r="C34" s="12"/>
+      <c r="D34" s="12"/>
+      <c r="E34" s="12"/>
+      <c r="F34" s="12"/>
+      <c r="G34" s="12"/>
+      <c r="H34" s="12"/>
+      <c r="I34" s="12"/>
+      <c r="J34" s="12"/>
+    </row>
+    <row r="35" spans="1:10" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A35" s="8" t="s">
+        <v>443</v>
+      </c>
+      <c r="B35" s="12"/>
+      <c r="C35" s="12"/>
+      <c r="D35" s="12"/>
+      <c r="E35" s="12"/>
+      <c r="F35" s="12"/>
+      <c r="G35" s="12"/>
+      <c r="H35" s="12"/>
+      <c r="I35" s="12"/>
+      <c r="J35" s="12"/>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="B31:J31"/>
+    <mergeCell ref="B32:J32"/>
+    <mergeCell ref="B33:J33"/>
+    <mergeCell ref="B34:J34"/>
+    <mergeCell ref="B35:J35"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CB17B1A6-CBE5-4654-A4B3-5FD415336E73}">
+  <sheetPr>
+    <tabColor rgb="FFC00000"/>
+  </sheetPr>
+  <dimension ref="A1:J5"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="16" style="1" customWidth="1"/>
+    <col min="2" max="2" width="12" style="1" customWidth="1"/>
+    <col min="3" max="3" width="40" style="1" customWidth="1"/>
+    <col min="4" max="4" width="46" style="1" customWidth="1"/>
+    <col min="5" max="6" width="34" style="1" customWidth="1"/>
+    <col min="7" max="7" width="14" style="1" customWidth="1"/>
+    <col min="8" max="8" width="12" style="1" customWidth="1"/>
+    <col min="9" max="10" width="14" style="1" customWidth="1"/>
+    <col min="11" max="16384" width="8.7109375" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:10" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="5" t="s">
+        <v>477</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>476</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>475</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>474</v>
+      </c>
+      <c r="E1" s="5" t="s">
+        <v>473</v>
+      </c>
+      <c r="F1" s="5" t="s">
+        <v>472</v>
+      </c>
+      <c r="G1" s="5" t="s">
+        <v>471</v>
+      </c>
+      <c r="H1" s="6" t="s">
+        <v>470</v>
+      </c>
+      <c r="I1" s="6" t="s">
+        <v>469</v>
+      </c>
+      <c r="J1" s="6" t="s">
+        <v>468</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A2" s="2"/>
+      <c r="B2" s="2"/>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+      <c r="G2" s="2"/>
+      <c r="H2" s="2"/>
+      <c r="I2" s="2"/>
+      <c r="J2" s="2"/>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A3" s="2"/>
+      <c r="B3" s="2"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2"/>
+      <c r="F3" s="2"/>
+      <c r="G3" s="2"/>
+      <c r="H3" s="2"/>
+      <c r="I3" s="2"/>
+      <c r="J3" s="2"/>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A4" s="2"/>
+      <c r="B4" s="2"/>
+      <c r="C4" s="2"/>
+      <c r="D4" s="2"/>
+      <c r="E4" s="2"/>
+      <c r="F4" s="2"/>
+      <c r="G4" s="2"/>
+      <c r="H4" s="2"/>
+      <c r="I4" s="2"/>
+      <c r="J4" s="2"/>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A5" s="2"/>
+      <c r="B5" s="2"/>
+      <c r="C5" s="2"/>
+      <c r="D5" s="2"/>
+      <c r="E5" s="2"/>
+      <c r="F5" s="2"/>
+      <c r="G5" s="2"/>
+      <c r="H5" s="2"/>
+      <c r="I5" s="2"/>
+      <c r="J5" s="2"/>
+    </row>
+  </sheetData>
+  <dataValidations count="2">
+    <dataValidation type="list" allowBlank="1" sqref="G2:G298" xr:uid="{00000000-0002-0000-0300-000000000000}">
+      <formula1>"Critical,High,Medium,Low"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" sqref="I2:I298" xr:uid="{00000000-0002-0000-0300-000001000000}">
+      <formula1>"Mới,Đang sửa,Đã sửa,Đã retest đạt,Retest lỗi lại"</formula1>
+      <formula2>0</formula2>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+</worksheet>
 </file>
</xml_diff>